<commit_message>
Files and minor edits for initial fitting of solana data
</commit_message>
<xml_diff>
--- a/solana-inputs/parameters_solana_exp.xlsx
+++ b/solana-inputs/parameters_solana_exp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limpo\SolarDynamics-code\HelioSoil-FS\solana-inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B7003B-0DDD-4088-8B03-A15682F44170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9DB40BD-7CEC-474D-8A9F-9EE10A3B32DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -225,9 +225,6 @@
     <t>Either "geometry" or "mie". If the latter, you need to supply a Source_Intensity tab in the simulation inputs</t>
   </si>
   <si>
-    <t>mie</t>
-  </si>
-  <si>
     <t>nominal_reflectance</t>
   </si>
   <si>
@@ -238,6 +235,9 @@
   </si>
   <si>
     <t>*elevation = 221 m at center of power block per google earth</t>
+  </si>
+  <si>
+    <t>geometry</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1114,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -1131,7 +1131,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1423,7 +1423,7 @@
         <v>62</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D27" t="s">
         <v>63</v>
@@ -1431,13 +1431,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B28">
         <v>0.94</v>
       </c>
       <c r="D28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>